<commit_message>
Update README.md text, example data, and example property outputs; remove item column from example parts list Excel data
</commit_message>
<xml_diff>
--- a/Example/Parts List.xlsx
+++ b/Example/Parts List.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t xml:space="preserve">PN</t>
   </si>
@@ -43,9 +43,6 @@
     <t xml:space="preserve">Pkg Price</t>
   </si>
   <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
     <t xml:space="preserve">SK1001-01</t>
   </si>
   <si>
@@ -59,9 +56,6 @@
   </si>
   <si>
     <t xml:space="preserve">BRX-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part</t>
   </si>
   <si>
     <t xml:space="preserve">SK1002-01</t>
@@ -487,7 +481,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.15"/>
@@ -497,6 +491,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16382" style="0" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -522,25 +517,22 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>1</v>
@@ -548,25 +540,22 @@
       <c r="G2" s="3" t="n">
         <v>67.95</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>1</v>
@@ -574,25 +563,22 @@
       <c r="G3" s="3" t="n">
         <v>28.95</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>1</v>
@@ -600,25 +586,22 @@
       <c r="G4" s="3" t="n">
         <v>3.49</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>8</v>
@@ -626,25 +609,22 @@
       <c r="G5" s="3" t="n">
         <v>44.95</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>25</v>
@@ -652,25 +632,22 @@
       <c r="G6" s="3" t="n">
         <v>12.49</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>25</v>
@@ -678,34 +655,28 @@
       <c r="G7" s="3" t="n">
         <v>9.89</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>8.95</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>